<commit_message>
feat(fasttrack): club 3 new onboarded tenants into FastTrack Excel sheet (141 total)
</commit_message>
<xml_diff>
--- a/Friendly_Space_PG_FastTrack_Import_Ready.xlsx
+++ b/Friendly_Space_PG_FastTrack_Import_Ready.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="FastTrack Import Roster" sheetId="1" r:id="rId1"/>
+    <sheet name="Friendly_Space_PG_FastTrack" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,24 +397,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P139"/>
+  <dimension ref="A1:P142"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="27.83203125" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="23.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="17.83203125" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" customWidth="1"/>
     <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="22.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="24.83203125" customWidth="1"/>
+    <col min="13" max="13" width="17.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="29.83203125" customWidth="1"/>
+    <col min="16" max="16" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,19 +472,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>GA</v>
+        <v>101</v>
       </c>
       <c r="C2" t="str">
-        <v>PG Management</v>
+        <v>Mrityunjay Kumar</v>
       </c>
       <c r="D2" t="str">
         <v>Bed A</v>
       </c>
       <c r="E2" t="str">
-        <v>7090803339</v>
+        <v>9999610585</v>
       </c>
       <c r="F2" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G2" t="str">
         <v/>
@@ -496,16 +496,16 @@
         <v>Tenant</v>
       </c>
       <c r="J2" t="str">
-        <v>01 Nov 2026</v>
+        <v>07 Sep 2026</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>3000</v>
       </c>
       <c r="M2" t="str">
-        <v>No (Due)</v>
+        <v>Yes (Paid)</v>
       </c>
       <c r="N2" t="str">
         <v>Yes (Paid)</v>
@@ -525,13 +525,13 @@
         <v>101</v>
       </c>
       <c r="C3" t="str">
-        <v>Mrityunjay Kumar</v>
+        <v>Rakshit Kumar</v>
       </c>
       <c r="D3" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E3" t="str">
-        <v>9999610585</v>
+        <v>9353822382</v>
       </c>
       <c r="F3" t="str">
         <v>2-Sharing</v>
@@ -546,13 +546,13 @@
         <v>Tenant</v>
       </c>
       <c r="J3" t="str">
-        <v>07 Sep 2026</v>
+        <v>01 May 2026</v>
       </c>
       <c r="K3">
         <v>10000</v>
       </c>
       <c r="L3">
-        <v>3000</v>
+        <v>1</v>
       </c>
       <c r="M3" t="str">
         <v>Yes (Paid)</v>
@@ -564,7 +564,7 @@
         <v>0</v>
       </c>
       <c r="P3" t="str">
-        <v/>
+        <v>KA02LK5689</v>
       </c>
     </row>
     <row r="4">
@@ -572,19 +572,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C4" t="str">
-        <v>Rakshit Kumar</v>
+        <v xml:space="preserve">Sai Ram </v>
       </c>
       <c r="D4" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E4" t="str">
-        <v>9353822382</v>
+        <v>9347209728</v>
       </c>
       <c r="F4" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G4" t="str">
         <v/>
@@ -596,7 +596,7 @@
         <v>Tenant</v>
       </c>
       <c r="J4" t="str">
-        <v>01 May 2026</v>
+        <v>06 Oct 2026</v>
       </c>
       <c r="K4">
         <v>10000</v>
@@ -614,7 +614,7 @@
         <v>0</v>
       </c>
       <c r="P4" t="str">
-        <v>KA02LK5689</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -622,19 +622,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C5" t="str">
-        <v xml:space="preserve">Sai Ram </v>
+        <v>Sai mahesh</v>
       </c>
       <c r="D5" t="str">
         <v>Bed A</v>
       </c>
       <c r="E5" t="str">
-        <v>9347209728</v>
+        <v>9347286321</v>
       </c>
       <c r="F5" t="str">
-        <v>Single</v>
+        <v>3-Sharing</v>
       </c>
       <c r="G5" t="str">
         <v/>
@@ -646,10 +646,10 @@
         <v>Tenant</v>
       </c>
       <c r="J5" t="str">
-        <v>06 Oct 2026</v>
+        <v>01 Apr 2026</v>
       </c>
       <c r="K5">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="L5">
         <v>1</v>
@@ -664,7 +664,7 @@
         <v>0</v>
       </c>
       <c r="P5" t="str">
-        <v/>
+        <v>AP16EA0782</v>
       </c>
     </row>
     <row r="6">
@@ -675,13 +675,13 @@
         <v>103</v>
       </c>
       <c r="C6" t="str">
-        <v>Sai mahesh</v>
+        <v>Pramod Kumar</v>
       </c>
       <c r="D6" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E6" t="str">
-        <v>9347286321</v>
+        <v>9030254092</v>
       </c>
       <c r="F6" t="str">
         <v>3-Sharing</v>
@@ -696,7 +696,7 @@
         <v>Tenant</v>
       </c>
       <c r="J6" t="str">
-        <v>01 Apr 2026</v>
+        <v>19 Aug 2026</v>
       </c>
       <c r="K6">
         <v>8000</v>
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
       <c r="P6" t="str">
-        <v>AP16EA0782</v>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -725,13 +725,13 @@
         <v>103</v>
       </c>
       <c r="C7" t="str">
-        <v>Pramod Kumar</v>
+        <v>Subramanyam</v>
       </c>
       <c r="D7" t="str">
-        <v>Bed B</v>
+        <v>Bed C</v>
       </c>
       <c r="E7" t="str">
-        <v>9030254092</v>
+        <v>8523868987</v>
       </c>
       <c r="F7" t="str">
         <v>3-Sharing</v>
@@ -746,10 +746,10 @@
         <v>Tenant</v>
       </c>
       <c r="J7" t="str">
-        <v>19 Aug 2026</v>
+        <v>04 Aug 2026</v>
       </c>
       <c r="K7">
-        <v>8000</v>
+        <v>8300</v>
       </c>
       <c r="L7">
         <v>1</v>
@@ -764,7 +764,7 @@
         <v>0</v>
       </c>
       <c r="P7" t="str">
-        <v/>
+        <v>AP37DE9897</v>
       </c>
     </row>
     <row r="8">
@@ -772,19 +772,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C8" t="str">
-        <v>Subramanyam</v>
+        <v>Sudharshan B</v>
       </c>
       <c r="D8" t="str">
-        <v>Bed C</v>
+        <v>Bed A</v>
       </c>
       <c r="E8" t="str">
-        <v>8523868987</v>
+        <v>9080101414</v>
       </c>
       <c r="F8" t="str">
-        <v>3-Sharing</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -796,10 +796,10 @@
         <v>Tenant</v>
       </c>
       <c r="J8" t="str">
-        <v>04 Aug 2026</v>
+        <v>09 Jul 2026</v>
       </c>
       <c r="K8">
-        <v>8300</v>
+        <v>10900</v>
       </c>
       <c r="L8">
         <v>1</v>
@@ -814,7 +814,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="str">
-        <v>AP37DE9897</v>
+        <v>TN83Y8974</v>
       </c>
     </row>
     <row r="9">
@@ -825,13 +825,13 @@
         <v>104</v>
       </c>
       <c r="C9" t="str">
-        <v>Sudharshan B</v>
+        <v>J Dharmesh</v>
       </c>
       <c r="D9" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E9" t="str">
-        <v>9080101414</v>
+        <v>9585431847</v>
       </c>
       <c r="F9" t="str">
         <v>2-Sharing</v>
@@ -846,10 +846,10 @@
         <v>Tenant</v>
       </c>
       <c r="J9" t="str">
-        <v>09 Jul 2026</v>
+        <v>18 Jul 2026</v>
       </c>
       <c r="K9">
-        <v>10900</v>
+        <v>10500</v>
       </c>
       <c r="L9">
         <v>1</v>
@@ -864,7 +864,7 @@
         <v>0</v>
       </c>
       <c r="P9" t="str">
-        <v>TN83Y8974</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -872,19 +872,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C10" t="str">
-        <v>J Dharmesh</v>
+        <v>kiran / Savithri</v>
       </c>
       <c r="D10" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E10" t="str">
-        <v>9585431847</v>
+        <v>8754245423</v>
       </c>
       <c r="F10" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -896,10 +896,10 @@
         <v>Tenant</v>
       </c>
       <c r="J10" t="str">
-        <v>18 Jul 2026</v>
+        <v>05 Jan 2026</v>
       </c>
       <c r="K10">
-        <v>10500</v>
+        <v>22000</v>
       </c>
       <c r="L10">
         <v>1</v>
@@ -922,22 +922,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C11" t="str">
-        <v>kiran / Savithri</v>
+        <v>Pavan</v>
       </c>
       <c r="D11" t="str">
         <v>Bed A</v>
       </c>
       <c r="E11" t="str">
-        <v>8754245423</v>
+        <v>6303333733</v>
       </c>
       <c r="F11" t="str">
         <v>Single</v>
       </c>
       <c r="G11" t="str">
-        <v/>
+        <v>Qualcomm</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -946,25 +946,25 @@
         <v>Tenant</v>
       </c>
       <c r="J11" t="str">
-        <v>05 Jan 2026</v>
+        <v>31 Oct 2026</v>
       </c>
       <c r="K11">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="L11">
-        <v>1</v>
+        <v>5000</v>
       </c>
       <c r="M11" t="str">
-        <v>Yes (Paid)</v>
+        <v>No (Due)</v>
       </c>
       <c r="N11" t="str">
-        <v>Yes (Paid)</v>
+        <v>No (Due)</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11" t="str">
-        <v/>
+        <v>AP39 QT 5625</v>
       </c>
     </row>
     <row r="12">
@@ -2984,7 +2984,7 @@
         <v>8431197622</v>
       </c>
       <c r="F52" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G52" t="str">
         <v>Canarys Automations</v>
@@ -3022,22 +3022,22 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C53" t="str">
-        <v>Priya Krishna</v>
+        <v>AMIT Raj Singh</v>
       </c>
       <c r="D53" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E53" t="str">
-        <v>8142058398</v>
+        <v>8630465075</v>
       </c>
       <c r="F53" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G53" t="str">
-        <v/>
+        <v>Unemployed</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -3046,13 +3046,13 @@
         <v>Tenant</v>
       </c>
       <c r="J53" t="str">
-        <v>05 Jan 2026</v>
+        <v>31 Oct 2026</v>
       </c>
       <c r="K53">
-        <v>11000</v>
+        <v>10000</v>
       </c>
       <c r="L53">
-        <v>1</v>
+        <v>2000</v>
       </c>
       <c r="M53" t="str">
         <v>Yes (Paid)</v>
@@ -3072,16 +3072,16 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C54" t="str">
-        <v>Thungam Narendra</v>
+        <v>Priya Krishna</v>
       </c>
       <c r="D54" t="str">
         <v>Bed A</v>
       </c>
       <c r="E54" t="str">
-        <v>9494891301</v>
+        <v>8142058398</v>
       </c>
       <c r="F54" t="str">
         <v>Single</v>
@@ -3096,10 +3096,10 @@
         <v>Tenant</v>
       </c>
       <c r="J54" t="str">
-        <v>01 Feb 2026</v>
+        <v>05 Jan 2026</v>
       </c>
       <c r="K54">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="L54">
         <v>1</v>
@@ -3122,19 +3122,19 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C55" t="str">
-        <v>Kapaka Ajay kumar</v>
+        <v>Thungam Narendra</v>
       </c>
       <c r="D55" t="str">
         <v>Bed A</v>
       </c>
       <c r="E55" t="str">
-        <v>7993681796</v>
+        <v>9494891301</v>
       </c>
       <c r="F55" t="str">
-        <v>3-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G55" t="str">
         <v/>
@@ -3146,10 +3146,10 @@
         <v>Tenant</v>
       </c>
       <c r="J55" t="str">
-        <v>04 Dec 2025</v>
+        <v>01 Feb 2026</v>
       </c>
       <c r="K55">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="L55">
         <v>1</v>
@@ -3175,13 +3175,13 @@
         <v>305</v>
       </c>
       <c r="C56" t="str">
-        <v>Umesh Chandra</v>
+        <v>Kapaka Ajay kumar</v>
       </c>
       <c r="D56" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E56" t="str">
-        <v>7995183073</v>
+        <v>7993681796</v>
       </c>
       <c r="F56" t="str">
         <v>3-Sharing</v>
@@ -3214,7 +3214,7 @@
         <v>0</v>
       </c>
       <c r="P56" t="str">
-        <v>AP37DP4560</v>
+        <v/>
       </c>
     </row>
     <row r="57">
@@ -3225,13 +3225,13 @@
         <v>305</v>
       </c>
       <c r="C57" t="str">
-        <v>Komala Aditya Ganesh</v>
+        <v>Umesh Chandra</v>
       </c>
       <c r="D57" t="str">
-        <v>Bed C</v>
+        <v>Bed B</v>
       </c>
       <c r="E57" t="str">
-        <v>7989268229</v>
+        <v>7995183073</v>
       </c>
       <c r="F57" t="str">
         <v>3-Sharing</v>
@@ -3264,7 +3264,7 @@
         <v>0</v>
       </c>
       <c r="P57" t="str">
-        <v/>
+        <v>AP37DP4560</v>
       </c>
     </row>
     <row r="58">
@@ -3272,22 +3272,22 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C58" t="str">
-        <v>Harish</v>
+        <v>Komala Aditya Ganesh</v>
       </c>
       <c r="D58" t="str">
-        <v>Bed A</v>
+        <v>Bed C</v>
       </c>
       <c r="E58" t="str">
-        <v>9342251506</v>
+        <v>7989268229</v>
       </c>
       <c r="F58" t="str">
-        <v>2-Sharing</v>
+        <v>3-Sharing</v>
       </c>
       <c r="G58" t="str">
-        <v>.</v>
+        <v/>
       </c>
       <c r="H58" t="str">
         <v/>
@@ -3296,13 +3296,13 @@
         <v>Tenant</v>
       </c>
       <c r="J58" t="str">
-        <v>29 Oct 2026</v>
+        <v>04 Dec 2025</v>
       </c>
       <c r="K58">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="L58">
-        <v>4500</v>
+        <v>1</v>
       </c>
       <c r="M58" t="str">
         <v>Yes (Paid)</v>
@@ -3325,19 +3325,19 @@
         <v>306</v>
       </c>
       <c r="C59" t="str">
-        <v>Bala chandar</v>
+        <v>Harish</v>
       </c>
       <c r="D59" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E59" t="str">
-        <v>9940407252</v>
+        <v>9342251506</v>
       </c>
       <c r="F59" t="str">
         <v>2-Sharing</v>
       </c>
       <c r="G59" t="str">
-        <v/>
+        <v>.</v>
       </c>
       <c r="H59" t="str">
         <v/>
@@ -3346,7 +3346,7 @@
         <v>Tenant</v>
       </c>
       <c r="J59" t="str">
-        <v>10 Sep 2026</v>
+        <v>29 Oct 2026</v>
       </c>
       <c r="K59">
         <v>10000</v>
@@ -3355,7 +3355,7 @@
         <v>4500</v>
       </c>
       <c r="M59" t="str">
-        <v>No (Due)</v>
+        <v>Yes (Paid)</v>
       </c>
       <c r="N59" t="str">
         <v>Yes (Paid)</v>
@@ -3372,19 +3372,19 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C60" t="str">
-        <v>Aditya Sanjay Raut</v>
+        <v>Bala chandar</v>
       </c>
       <c r="D60" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E60" t="str">
-        <v>8884872737</v>
+        <v>9940407252</v>
       </c>
       <c r="F60" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G60" t="str">
         <v/>
@@ -3396,16 +3396,16 @@
         <v>Tenant</v>
       </c>
       <c r="J60" t="str">
-        <v>03 Aug 2026</v>
+        <v>10 Sep 2026</v>
       </c>
       <c r="K60">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="L60">
-        <v>1</v>
+        <v>4500</v>
       </c>
       <c r="M60" t="str">
-        <v>Yes (Paid)</v>
+        <v>No (Due)</v>
       </c>
       <c r="N60" t="str">
         <v>Yes (Paid)</v>
@@ -3422,19 +3422,19 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C61" t="str">
-        <v>Bishnuprasad Nath</v>
+        <v>Aditya Sanjay Raut</v>
       </c>
       <c r="D61" t="str">
         <v>Bed A</v>
       </c>
       <c r="E61" t="str">
-        <v>7259317888</v>
+        <v>8884872737</v>
       </c>
       <c r="F61" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G61" t="str">
         <v/>
@@ -3446,10 +3446,10 @@
         <v>Tenant</v>
       </c>
       <c r="J61" t="str">
-        <v>08 Aug 2026</v>
+        <v>03 Aug 2026</v>
       </c>
       <c r="K61">
-        <v>11400</v>
+        <v>20000</v>
       </c>
       <c r="L61">
         <v>1</v>
@@ -3475,13 +3475,13 @@
         <v>308</v>
       </c>
       <c r="C62" t="str">
-        <v>Prasad Basavaraj Warad</v>
+        <v>Bishnuprasad Nath</v>
       </c>
       <c r="D62" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E62" t="str">
-        <v>9869301625</v>
+        <v>7259317888</v>
       </c>
       <c r="F62" t="str">
         <v>2-Sharing</v>
@@ -3496,10 +3496,10 @@
         <v>Tenant</v>
       </c>
       <c r="J62" t="str">
-        <v>16 Aug 2026</v>
+        <v>08 Aug 2026</v>
       </c>
       <c r="K62">
-        <v>11000</v>
+        <v>11400</v>
       </c>
       <c r="L62">
         <v>1</v>
@@ -3522,19 +3522,19 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C63" t="str">
-        <v>Y Bargav</v>
+        <v>Prasad Basavaraj Warad</v>
       </c>
       <c r="D63" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E63" t="str">
-        <v>7995236669</v>
+        <v>9869301625</v>
       </c>
       <c r="F63" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G63" t="str">
         <v/>
@@ -3546,10 +3546,10 @@
         <v>Tenant</v>
       </c>
       <c r="J63" t="str">
-        <v>09 Sep 2026</v>
+        <v>16 Aug 2026</v>
       </c>
       <c r="K63">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="L63">
         <v>1</v>
@@ -3572,16 +3572,16 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C64" t="str">
-        <v>Aproov Raj Tripati</v>
+        <v>Y Bargav</v>
       </c>
       <c r="D64" t="str">
         <v>Bed A</v>
       </c>
       <c r="E64" t="str">
-        <v>9616285086</v>
+        <v>7995236669</v>
       </c>
       <c r="F64" t="str">
         <v>Single</v>
@@ -3596,10 +3596,10 @@
         <v>Tenant</v>
       </c>
       <c r="J64" t="str">
-        <v>31 Jul 2026</v>
+        <v>09 Sep 2026</v>
       </c>
       <c r="K64">
-        <v>21000</v>
+        <v>10000</v>
       </c>
       <c r="L64">
         <v>1</v>
@@ -3622,16 +3622,16 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C65" t="str">
-        <v>Ajinkya chandrakant</v>
+        <v>Aproov Raj Tripati</v>
       </c>
       <c r="D65" t="str">
         <v>Bed A</v>
       </c>
       <c r="E65" t="str">
-        <v>8308841485</v>
+        <v>9616285086</v>
       </c>
       <c r="F65" t="str">
         <v>Single</v>
@@ -3646,10 +3646,10 @@
         <v>Tenant</v>
       </c>
       <c r="J65" t="str">
-        <v>31 Jan 2026</v>
+        <v>31 Jul 2026</v>
       </c>
       <c r="K65">
-        <v>18000</v>
+        <v>21000</v>
       </c>
       <c r="L65">
         <v>1</v>
@@ -3672,19 +3672,19 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C66" t="str">
-        <v>Kaipu Nagarjuna Reddy</v>
+        <v>Ajinkya chandrakant</v>
       </c>
       <c r="D66" t="str">
         <v>Bed A</v>
       </c>
       <c r="E66" t="str">
-        <v>8464078907</v>
+        <v>8308841485</v>
       </c>
       <c r="F66" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G66" t="str">
         <v/>
@@ -3696,10 +3696,10 @@
         <v>Tenant</v>
       </c>
       <c r="J66" t="str">
-        <v>08 Apr 2026</v>
+        <v>31 Jan 2026</v>
       </c>
       <c r="K66">
-        <v>10000</v>
+        <v>18000</v>
       </c>
       <c r="L66">
         <v>1</v>
@@ -3725,13 +3725,13 @@
         <v>314</v>
       </c>
       <c r="C67" t="str">
-        <v>Praveen Meena</v>
+        <v>Kaipu Nagarjuna Reddy</v>
       </c>
       <c r="D67" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E67" t="str">
-        <v>6263721191</v>
+        <v>8464078907</v>
       </c>
       <c r="F67" t="str">
         <v>2-Sharing</v>
@@ -3746,10 +3746,10 @@
         <v>Tenant</v>
       </c>
       <c r="J67" t="str">
-        <v>01 Apr 2026</v>
+        <v>08 Apr 2026</v>
       </c>
       <c r="K67">
-        <v>10500</v>
+        <v>10000</v>
       </c>
       <c r="L67">
         <v>1</v>
@@ -3772,16 +3772,16 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>401</v>
+        <v>314</v>
       </c>
       <c r="C68" t="str">
-        <v>Gaurav Vilas Autade</v>
+        <v>Praveen Meena</v>
       </c>
       <c r="D68" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E68" t="str">
-        <v>8108840046</v>
+        <v>6263721191</v>
       </c>
       <c r="F68" t="str">
         <v>2-Sharing</v>
@@ -3796,10 +3796,10 @@
         <v>Tenant</v>
       </c>
       <c r="J68" t="str">
-        <v>04 Nov 2025</v>
+        <v>01 Apr 2026</v>
       </c>
       <c r="K68">
-        <v>12000</v>
+        <v>10500</v>
       </c>
       <c r="L68">
         <v>1</v>
@@ -3825,13 +3825,13 @@
         <v>401</v>
       </c>
       <c r="C69" t="str">
-        <v>Karthik Nair</v>
+        <v>Gaurav Vilas Autade</v>
       </c>
       <c r="D69" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E69" t="str">
-        <v>9696122374</v>
+        <v>8108840046</v>
       </c>
       <c r="F69" t="str">
         <v>2-Sharing</v>
@@ -3846,7 +3846,7 @@
         <v>Tenant</v>
       </c>
       <c r="J69" t="str">
-        <v>04 Sep 2026</v>
+        <v>04 Nov 2025</v>
       </c>
       <c r="K69">
         <v>12000</v>
@@ -3872,16 +3872,16 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C70" t="str">
-        <v>Soumydip Das</v>
+        <v>Karthik Nair</v>
       </c>
       <c r="D70" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E70" t="str">
-        <v>9954954950</v>
+        <v>9696122374</v>
       </c>
       <c r="F70" t="str">
         <v>2-Sharing</v>
@@ -3896,10 +3896,10 @@
         <v>Tenant</v>
       </c>
       <c r="J70" t="str">
-        <v>10 Jan 2026</v>
+        <v>04 Sep 2026</v>
       </c>
       <c r="K70">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="L70">
         <v>1</v>
@@ -3925,13 +3925,13 @@
         <v>402</v>
       </c>
       <c r="C71" t="str">
-        <v>Uditya Raj</v>
+        <v>Soumydip Das</v>
       </c>
       <c r="D71" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E71" t="str">
-        <v>6299625674</v>
+        <v>9954954950</v>
       </c>
       <c r="F71" t="str">
         <v>2-Sharing</v>
@@ -3972,19 +3972,19 @@
         <v>71</v>
       </c>
       <c r="B72" t="str">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C72" t="str">
-        <v>Rachaputi Lilithkumar</v>
+        <v>Uditya Raj</v>
       </c>
       <c r="D72" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E72" t="str">
-        <v>9177250177</v>
+        <v>6299625674</v>
       </c>
       <c r="F72" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G72" t="str">
         <v/>
@@ -3996,10 +3996,10 @@
         <v>Tenant</v>
       </c>
       <c r="J72" t="str">
-        <v>16 Jan 2026</v>
+        <v>10 Jan 2026</v>
       </c>
       <c r="K72">
-        <v>11000</v>
+        <v>10000</v>
       </c>
       <c r="L72">
         <v>1</v>
@@ -4022,19 +4022,19 @@
         <v>72</v>
       </c>
       <c r="B73" t="str">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C73" t="str">
-        <v>Ashwin</v>
+        <v>Rachaputi Lilithkumar</v>
       </c>
       <c r="D73" t="str">
         <v>Bed A</v>
       </c>
       <c r="E73" t="str">
-        <v>9025037259</v>
+        <v>9177250177</v>
       </c>
       <c r="F73" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G73" t="str">
         <v/>
@@ -4046,10 +4046,10 @@
         <v>Tenant</v>
       </c>
       <c r="J73" t="str">
-        <v>14 Aug 2026</v>
+        <v>16 Jan 2026</v>
       </c>
       <c r="K73">
-        <v>10500</v>
+        <v>11000</v>
       </c>
       <c r="L73">
         <v>1</v>
@@ -4075,13 +4075,13 @@
         <v>404</v>
       </c>
       <c r="C74" t="str">
-        <v>M Kamalesh</v>
+        <v>Ashwin</v>
       </c>
       <c r="D74" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E74" t="str">
-        <v>8148310238</v>
+        <v>9025037259</v>
       </c>
       <c r="F74" t="str">
         <v>2-Sharing</v>
@@ -4096,10 +4096,10 @@
         <v>Tenant</v>
       </c>
       <c r="J74" t="str">
-        <v>09 Aug 2026</v>
+        <v>14 Aug 2026</v>
       </c>
       <c r="K74">
-        <v>10900</v>
+        <v>10500</v>
       </c>
       <c r="L74">
         <v>1</v>
@@ -4122,19 +4122,19 @@
         <v>74</v>
       </c>
       <c r="B75" t="str">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C75" t="str">
-        <v>Sham Sundar</v>
+        <v>M Kamalesh</v>
       </c>
       <c r="D75" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E75" t="str">
-        <v>7075723054</v>
+        <v>8148310238</v>
       </c>
       <c r="F75" t="str">
-        <v>3-Sharing</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G75" t="str">
         <v/>
@@ -4146,10 +4146,10 @@
         <v>Tenant</v>
       </c>
       <c r="J75" t="str">
-        <v>01 Nov 2025</v>
+        <v>09 Aug 2026</v>
       </c>
       <c r="K75">
-        <v>8000</v>
+        <v>10900</v>
       </c>
       <c r="L75">
         <v>1</v>
@@ -4175,13 +4175,13 @@
         <v>405</v>
       </c>
       <c r="C76" t="str">
-        <v>Maneesh</v>
+        <v>Sham Sundar</v>
       </c>
       <c r="D76" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E76" t="str">
-        <v>8247682541</v>
+        <v>7075723054</v>
       </c>
       <c r="F76" t="str">
         <v>3-Sharing</v>
@@ -4202,7 +4202,7 @@
         <v>8000</v>
       </c>
       <c r="L76">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M76" t="str">
         <v>Yes (Paid)</v>
@@ -4214,7 +4214,7 @@
         <v>0</v>
       </c>
       <c r="P76" t="str">
-        <v>AP04AY3076</v>
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -4225,13 +4225,13 @@
         <v>405</v>
       </c>
       <c r="C77" t="str">
-        <v>Kaif</v>
+        <v>Maneesh</v>
       </c>
       <c r="D77" t="str">
-        <v>Bed C</v>
+        <v>Bed B</v>
       </c>
       <c r="E77" t="str">
-        <v>9121205990</v>
+        <v>8247682541</v>
       </c>
       <c r="F77" t="str">
         <v>3-Sharing</v>
@@ -4252,7 +4252,7 @@
         <v>8000</v>
       </c>
       <c r="L77">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M77" t="str">
         <v>Yes (Paid)</v>
@@ -4264,7 +4264,7 @@
         <v>0</v>
       </c>
       <c r="P77" t="str">
-        <v/>
+        <v>AP04AY3076</v>
       </c>
     </row>
     <row r="78">
@@ -4272,19 +4272,19 @@
         <v>77</v>
       </c>
       <c r="B78" t="str">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C78" t="str">
-        <v>Animesh Panda</v>
+        <v>Kaif</v>
       </c>
       <c r="D78" t="str">
-        <v>Bed A</v>
+        <v>Bed C</v>
       </c>
       <c r="E78" t="str">
-        <v>8093818285</v>
+        <v>9121205990</v>
       </c>
       <c r="F78" t="str">
-        <v>Single</v>
+        <v>3-Sharing</v>
       </c>
       <c r="G78" t="str">
         <v/>
@@ -4296,10 +4296,10 @@
         <v>Tenant</v>
       </c>
       <c r="J78" t="str">
-        <v>22 Mar 2026</v>
+        <v>01 Nov 2025</v>
       </c>
       <c r="K78">
-        <v>19000</v>
+        <v>8000</v>
       </c>
       <c r="L78">
         <v>1</v>
@@ -4322,16 +4322,16 @@
         <v>78</v>
       </c>
       <c r="B79" t="str">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C79" t="str">
-        <v>Aditya Hegde</v>
+        <v>Animesh Panda</v>
       </c>
       <c r="D79" t="str">
         <v>Bed A</v>
       </c>
       <c r="E79" t="str">
-        <v>8792437717</v>
+        <v>8093818285</v>
       </c>
       <c r="F79" t="str">
         <v>Single</v>
@@ -4346,10 +4346,10 @@
         <v>Tenant</v>
       </c>
       <c r="J79" t="str">
-        <v>02 Jan 2026</v>
+        <v>22 Mar 2026</v>
       </c>
       <c r="K79">
-        <v>18000</v>
+        <v>19000</v>
       </c>
       <c r="L79">
         <v>1</v>
@@ -4372,19 +4372,19 @@
         <v>79</v>
       </c>
       <c r="B80" t="str">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C80" t="str">
-        <v>Priyaraj sunny</v>
+        <v>Aditya Hegde</v>
       </c>
       <c r="D80" t="str">
         <v>Bed A</v>
       </c>
       <c r="E80" t="str">
-        <v>7001741489</v>
+        <v>8792437717</v>
       </c>
       <c r="F80" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G80" t="str">
         <v/>
@@ -4396,10 +4396,10 @@
         <v>Tenant</v>
       </c>
       <c r="J80" t="str">
-        <v>01 Dec 2025</v>
+        <v>02 Jan 2026</v>
       </c>
       <c r="K80">
-        <v>10000</v>
+        <v>18000</v>
       </c>
       <c r="L80">
         <v>1</v>
@@ -4414,7 +4414,7 @@
         <v>0</v>
       </c>
       <c r="P80" t="str">
-        <v>TN07DK2268</v>
+        <v/>
       </c>
     </row>
     <row r="81">
@@ -4425,13 +4425,13 @@
         <v>408</v>
       </c>
       <c r="C81" t="str">
-        <v>Gammath Karthik</v>
+        <v>Priyaraj sunny</v>
       </c>
       <c r="D81" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E81" t="str">
-        <v>9014990138</v>
+        <v>7001741489</v>
       </c>
       <c r="F81" t="str">
         <v>2-Sharing</v>
@@ -4446,7 +4446,7 @@
         <v>Tenant</v>
       </c>
       <c r="J81" t="str">
-        <v>02 Jan 2026</v>
+        <v>01 Dec 2025</v>
       </c>
       <c r="K81">
         <v>10000</v>
@@ -4464,7 +4464,7 @@
         <v>0</v>
       </c>
       <c r="P81" t="str">
-        <v/>
+        <v>TN07DK2268</v>
       </c>
     </row>
     <row r="82">
@@ -4472,19 +4472,19 @@
         <v>81</v>
       </c>
       <c r="B82" t="str">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C82" t="str">
-        <v>Soumya Ranjan jeda</v>
+        <v>Gammath Karthik</v>
       </c>
       <c r="D82" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E82" t="str">
-        <v>9051728176</v>
+        <v>9014990138</v>
       </c>
       <c r="F82" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G82" t="str">
         <v/>
@@ -4496,10 +4496,10 @@
         <v>Tenant</v>
       </c>
       <c r="J82" t="str">
-        <v>01 Feb 2026</v>
+        <v>02 Jan 2026</v>
       </c>
       <c r="K82">
-        <v>19500</v>
+        <v>10000</v>
       </c>
       <c r="L82">
         <v>1</v>
@@ -4514,7 +4514,7 @@
         <v>0</v>
       </c>
       <c r="P82" t="str">
-        <v>KA20HF7375</v>
+        <v/>
       </c>
     </row>
     <row r="83">
@@ -4522,16 +4522,16 @@
         <v>82</v>
       </c>
       <c r="B83" t="str">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C83" t="str">
-        <v>305 Umesh Friend</v>
+        <v>Soumya Ranjan jeda</v>
       </c>
       <c r="D83" t="str">
         <v>Bed A</v>
       </c>
       <c r="E83" t="str">
-        <v>9876543210</v>
+        <v>9051728176</v>
       </c>
       <c r="F83" t="str">
         <v>Single</v>
@@ -4546,10 +4546,10 @@
         <v>Tenant</v>
       </c>
       <c r="J83" t="str">
-        <v>06 Oct 2026</v>
+        <v>01 Feb 2026</v>
       </c>
       <c r="K83">
-        <v>16500</v>
+        <v>19500</v>
       </c>
       <c r="L83">
         <v>1</v>
@@ -4564,7 +4564,7 @@
         <v>0</v>
       </c>
       <c r="P83" t="str">
-        <v/>
+        <v>KA20HF7375</v>
       </c>
     </row>
     <row r="84">
@@ -4572,19 +4572,19 @@
         <v>83</v>
       </c>
       <c r="B84" t="str">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C84" t="str">
-        <v>kiran</v>
+        <v>305 Umesh Friend</v>
       </c>
       <c r="D84" t="str">
         <v>Bed A</v>
       </c>
       <c r="E84" t="str">
-        <v>9701001900</v>
+        <v>9876543210</v>
       </c>
       <c r="F84" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G84" t="str">
         <v/>
@@ -4596,10 +4596,10 @@
         <v>Tenant</v>
       </c>
       <c r="J84" t="str">
-        <v>12 Oct 2026</v>
+        <v>06 Oct 2026</v>
       </c>
       <c r="K84">
-        <v>11000</v>
+        <v>16500</v>
       </c>
       <c r="L84">
         <v>1</v>
@@ -4625,13 +4625,13 @@
         <v>411</v>
       </c>
       <c r="C85" t="str">
-        <v>Mohith</v>
+        <v>kiran</v>
       </c>
       <c r="D85" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E85" t="str">
-        <v>9610152365</v>
+        <v>9701001900</v>
       </c>
       <c r="F85" t="str">
         <v>2-Sharing</v>
@@ -4646,7 +4646,7 @@
         <v>Tenant</v>
       </c>
       <c r="J85" t="str">
-        <v>29 Aug 2026</v>
+        <v>12 Oct 2026</v>
       </c>
       <c r="K85">
         <v>11000</v>
@@ -4672,16 +4672,16 @@
         <v>85</v>
       </c>
       <c r="B86" t="str">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C86" t="str">
-        <v>Mohammed Saiful</v>
+        <v>Mohith</v>
       </c>
       <c r="D86" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E86" t="str">
-        <v>7548890354</v>
+        <v>9610152365</v>
       </c>
       <c r="F86" t="str">
         <v>2-Sharing</v>
@@ -4696,10 +4696,10 @@
         <v>Tenant</v>
       </c>
       <c r="J86" t="str">
-        <v>09 Aug 2026</v>
+        <v>29 Aug 2026</v>
       </c>
       <c r="K86">
-        <v>10500</v>
+        <v>11000</v>
       </c>
       <c r="L86">
         <v>1</v>
@@ -4725,13 +4725,13 @@
         <v>412</v>
       </c>
       <c r="C87" t="str">
-        <v>Mithun Hari K</v>
+        <v>Mohammed Saiful</v>
       </c>
       <c r="D87" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E87" t="str">
-        <v>9894865943</v>
+        <v>7548890354</v>
       </c>
       <c r="F87" t="str">
         <v>2-Sharing</v>
@@ -4772,19 +4772,19 @@
         <v>87</v>
       </c>
       <c r="B88" t="str">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C88" t="str">
-        <v>Dilip Kumar N</v>
+        <v>Mithun Hari K</v>
       </c>
       <c r="D88" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E88" t="str">
-        <v>9632101301</v>
+        <v>9894865943</v>
       </c>
       <c r="F88" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G88" t="str">
         <v/>
@@ -4796,10 +4796,10 @@
         <v>Tenant</v>
       </c>
       <c r="J88" t="str">
-        <v>31 Jul 2026</v>
+        <v>09 Aug 2026</v>
       </c>
       <c r="K88">
-        <v>18000</v>
+        <v>10500</v>
       </c>
       <c r="L88">
         <v>1</v>
@@ -4822,19 +4822,19 @@
         <v>88</v>
       </c>
       <c r="B89" t="str">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C89" t="str">
-        <v>Pranjal Avasthi</v>
+        <v>Dilip Kumar N</v>
       </c>
       <c r="D89" t="str">
         <v>Bed A</v>
       </c>
       <c r="E89" t="str">
-        <v>9696073285</v>
+        <v>9632101301</v>
       </c>
       <c r="F89" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G89" t="str">
         <v/>
@@ -4846,10 +4846,10 @@
         <v>Tenant</v>
       </c>
       <c r="J89" t="str">
-        <v>05 Jan 2026</v>
+        <v>31 Jul 2026</v>
       </c>
       <c r="K89">
-        <v>10000</v>
+        <v>18000</v>
       </c>
       <c r="L89">
         <v>1</v>
@@ -4864,7 +4864,7 @@
         <v>0</v>
       </c>
       <c r="P89" t="str">
-        <v>UP32ML3430</v>
+        <v/>
       </c>
     </row>
     <row r="90">
@@ -4875,13 +4875,13 @@
         <v>414</v>
       </c>
       <c r="C90" t="str">
-        <v>Shruthi Sarovar</v>
+        <v>Pranjal Avasthi</v>
       </c>
       <c r="D90" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E90" t="str">
-        <v>9648061542</v>
+        <v>9696073285</v>
       </c>
       <c r="F90" t="str">
         <v>2-Sharing</v>
@@ -4896,7 +4896,7 @@
         <v>Tenant</v>
       </c>
       <c r="J90" t="str">
-        <v>27 Jun 2026</v>
+        <v>05 Jan 2026</v>
       </c>
       <c r="K90">
         <v>10000</v>
@@ -4914,7 +4914,7 @@
         <v>0</v>
       </c>
       <c r="P90" t="str">
-        <v/>
+        <v>UP32ML3430</v>
       </c>
     </row>
     <row r="91">
@@ -4922,19 +4922,19 @@
         <v>90</v>
       </c>
       <c r="B91" t="str">
-        <v>501</v>
+        <v>414</v>
       </c>
       <c r="C91" t="str">
-        <v>Vinayak</v>
+        <v>Shruthi Sarovar</v>
       </c>
       <c r="D91" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E91" t="str">
-        <v>7095050785</v>
+        <v>9648061542</v>
       </c>
       <c r="F91" t="str">
-        <v>3-Sharing</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G91" t="str">
         <v/>
@@ -4946,10 +4946,10 @@
         <v>Tenant</v>
       </c>
       <c r="J91" t="str">
-        <v>01 Feb 2026</v>
+        <v>27 Jun 2026</v>
       </c>
       <c r="K91">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="L91">
         <v>1</v>
@@ -4964,7 +4964,7 @@
         <v>0</v>
       </c>
       <c r="P91" t="str">
-        <v>KA51JH5800</v>
+        <v/>
       </c>
     </row>
     <row r="92">
@@ -4975,13 +4975,13 @@
         <v>501</v>
       </c>
       <c r="C92" t="str">
-        <v>Kumaran</v>
+        <v>Vinayak</v>
       </c>
       <c r="D92" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E92" t="str">
-        <v>8667493156</v>
+        <v>7095050785</v>
       </c>
       <c r="F92" t="str">
         <v>3-Sharing</v>
@@ -4996,7 +4996,7 @@
         <v>Tenant</v>
       </c>
       <c r="J92" t="str">
-        <v>01 Sep 2026</v>
+        <v>01 Feb 2026</v>
       </c>
       <c r="K92">
         <v>8000</v>
@@ -5014,7 +5014,7 @@
         <v>0</v>
       </c>
       <c r="P92" t="str">
-        <v/>
+        <v>KA51JH5800</v>
       </c>
     </row>
     <row r="93">
@@ -5025,13 +5025,13 @@
         <v>501</v>
       </c>
       <c r="C93" t="str">
-        <v>Naidu</v>
+        <v>Kumaran</v>
       </c>
       <c r="D93" t="str">
-        <v>Bed C</v>
+        <v>Bed B</v>
       </c>
       <c r="E93" t="str">
-        <v>8465954721</v>
+        <v>8667493156</v>
       </c>
       <c r="F93" t="str">
         <v>3-Sharing</v>
@@ -5046,7 +5046,7 @@
         <v>Tenant</v>
       </c>
       <c r="J93" t="str">
-        <v>18 Sep 2026</v>
+        <v>01 Sep 2026</v>
       </c>
       <c r="K93">
         <v>8000</v>
@@ -5072,19 +5072,19 @@
         <v>93</v>
       </c>
       <c r="B94" t="str">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C94" t="str">
-        <v>Sidharth Kaushik</v>
+        <v>Naidu</v>
       </c>
       <c r="D94" t="str">
-        <v>Bed A</v>
+        <v>Bed C</v>
       </c>
       <c r="E94" t="str">
-        <v>7903565045</v>
+        <v>8465954721</v>
       </c>
       <c r="F94" t="str">
-        <v>2-Sharing</v>
+        <v>3-Sharing</v>
       </c>
       <c r="G94" t="str">
         <v/>
@@ -5096,10 +5096,10 @@
         <v>Tenant</v>
       </c>
       <c r="J94" t="str">
-        <v>13 Dec 2025</v>
+        <v>18 Sep 2026</v>
       </c>
       <c r="K94">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="L94">
         <v>1</v>
@@ -5125,13 +5125,13 @@
         <v>502</v>
       </c>
       <c r="C95" t="str">
-        <v>Shivashankarn</v>
+        <v>Sidharth Kaushik</v>
       </c>
       <c r="D95" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E95" t="str">
-        <v>6379088395</v>
+        <v>7903565045</v>
       </c>
       <c r="F95" t="str">
         <v>2-Sharing</v>
@@ -5146,7 +5146,7 @@
         <v>Tenant</v>
       </c>
       <c r="J95" t="str">
-        <v>05 Jan 2026</v>
+        <v>13 Dec 2025</v>
       </c>
       <c r="K95">
         <v>10000</v>
@@ -5172,16 +5172,16 @@
         <v>95</v>
       </c>
       <c r="B96" t="str">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C96" t="str">
-        <v>Abhishek kumar Giri</v>
+        <v>Shivashankarn</v>
       </c>
       <c r="D96" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E96" t="str">
-        <v>8478896615</v>
+        <v>6379088395</v>
       </c>
       <c r="F96" t="str">
         <v>2-Sharing</v>
@@ -5196,7 +5196,7 @@
         <v>Tenant</v>
       </c>
       <c r="J96" t="str">
-        <v>28 Nov 2025</v>
+        <v>05 Jan 2026</v>
       </c>
       <c r="K96">
         <v>10000</v>
@@ -5225,13 +5225,13 @@
         <v>503</v>
       </c>
       <c r="C97" t="str">
-        <v>Hema venkat Ramesh</v>
+        <v>Abhishek kumar Giri</v>
       </c>
       <c r="D97" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E97" t="str">
-        <v>9206651295</v>
+        <v>8478896615</v>
       </c>
       <c r="F97" t="str">
         <v>2-Sharing</v>
@@ -5246,10 +5246,10 @@
         <v>Tenant</v>
       </c>
       <c r="J97" t="str">
-        <v>01 Dec 2025</v>
+        <v>28 Nov 2025</v>
       </c>
       <c r="K97">
-        <v>10400</v>
+        <v>10000</v>
       </c>
       <c r="L97">
         <v>1</v>
@@ -5264,7 +5264,7 @@
         <v>0</v>
       </c>
       <c r="P97" t="str">
-        <v>KA03KP4779</v>
+        <v/>
       </c>
     </row>
     <row r="98">
@@ -5272,19 +5272,19 @@
         <v>97</v>
       </c>
       <c r="B98" t="str">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C98" t="str">
-        <v>Kaushik</v>
+        <v>Hema venkat Ramesh</v>
       </c>
       <c r="D98" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E98" t="str">
-        <v>8105732597</v>
+        <v>9206651295</v>
       </c>
       <c r="F98" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G98" t="str">
         <v/>
@@ -5296,10 +5296,10 @@
         <v>Tenant</v>
       </c>
       <c r="J98" t="str">
-        <v>05 Jan 2026</v>
+        <v>01 Dec 2025</v>
       </c>
       <c r="K98">
-        <v>20000</v>
+        <v>10400</v>
       </c>
       <c r="L98">
         <v>1</v>
@@ -5314,7 +5314,7 @@
         <v>0</v>
       </c>
       <c r="P98" t="str">
-        <v>KA09HR3283</v>
+        <v>KA03KP4779</v>
       </c>
     </row>
     <row r="99">
@@ -5322,19 +5322,19 @@
         <v>98</v>
       </c>
       <c r="B99" t="str">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C99" t="str">
-        <v>Peniel Jacob Paul</v>
+        <v>Kaushik</v>
       </c>
       <c r="D99" t="str">
         <v>Bed A</v>
       </c>
       <c r="E99" t="str">
-        <v>7904060336</v>
+        <v>8105732597</v>
       </c>
       <c r="F99" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G99" t="str">
         <v/>
@@ -5346,10 +5346,10 @@
         <v>Tenant</v>
       </c>
       <c r="J99" t="str">
-        <v>01 Dec 2025</v>
+        <v>05 Jan 2026</v>
       </c>
       <c r="K99">
-        <v>12000</v>
+        <v>20000</v>
       </c>
       <c r="L99">
         <v>1</v>
@@ -5364,7 +5364,7 @@
         <v>0</v>
       </c>
       <c r="P99" t="str">
-        <v>KA01KK5927</v>
+        <v>KA09HR3283</v>
       </c>
     </row>
     <row r="100">
@@ -5375,13 +5375,13 @@
         <v>505</v>
       </c>
       <c r="C100" t="str">
-        <v>R Vignesh</v>
+        <v>Peniel Jacob Paul</v>
       </c>
       <c r="D100" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E100" t="str">
-        <v>9199355107</v>
+        <v>7904060336</v>
       </c>
       <c r="F100" t="str">
         <v>2-Sharing</v>
@@ -5396,7 +5396,7 @@
         <v>Tenant</v>
       </c>
       <c r="J100" t="str">
-        <v>05 Jan 2026</v>
+        <v>01 Dec 2025</v>
       </c>
       <c r="K100">
         <v>12000</v>
@@ -5414,7 +5414,7 @@
         <v>0</v>
       </c>
       <c r="P100" t="str">
-        <v>KA02JE6414</v>
+        <v>KA01KK5927</v>
       </c>
     </row>
     <row r="101">
@@ -5422,19 +5422,19 @@
         <v>100</v>
       </c>
       <c r="B101" t="str">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C101" t="str">
-        <v>Shoibul Houqa</v>
+        <v>R Vignesh</v>
       </c>
       <c r="D101" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E101" t="str">
-        <v>7829860087</v>
+        <v>9199355107</v>
       </c>
       <c r="F101" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G101" t="str">
         <v/>
@@ -5446,10 +5446,10 @@
         <v>Tenant</v>
       </c>
       <c r="J101" t="str">
-        <v>22 Oct 2026</v>
+        <v>05 Jan 2026</v>
       </c>
       <c r="K101">
-        <v>20000</v>
+        <v>12000</v>
       </c>
       <c r="L101">
         <v>1</v>
@@ -5464,7 +5464,7 @@
         <v>0</v>
       </c>
       <c r="P101" t="str">
-        <v/>
+        <v>KA02JE6414</v>
       </c>
     </row>
     <row r="102">
@@ -5472,16 +5472,16 @@
         <v>101</v>
       </c>
       <c r="B102" t="str">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C102" t="str">
-        <v>Aditya Gaunkar</v>
+        <v>Shoibul Houqa</v>
       </c>
       <c r="D102" t="str">
         <v>Bed A</v>
       </c>
       <c r="E102" t="str">
-        <v>8431547954</v>
+        <v>7829860087</v>
       </c>
       <c r="F102" t="str">
         <v>Single</v>
@@ -5496,10 +5496,10 @@
         <v>Tenant</v>
       </c>
       <c r="J102" t="str">
-        <v>01 Nov 2025</v>
+        <v>22 Oct 2026</v>
       </c>
       <c r="K102">
-        <v>19000</v>
+        <v>20000</v>
       </c>
       <c r="L102">
         <v>1</v>
@@ -5522,16 +5522,16 @@
         <v>102</v>
       </c>
       <c r="B103" t="str">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C103" t="str">
-        <v>Vidya poorna HS</v>
+        <v>Aditya Gaunkar</v>
       </c>
       <c r="D103" t="str">
         <v>Bed A</v>
       </c>
       <c r="E103" t="str">
-        <v>9663491347</v>
+        <v>8431547954</v>
       </c>
       <c r="F103" t="str">
         <v>Single</v>
@@ -5572,16 +5572,16 @@
         <v>103</v>
       </c>
       <c r="B104" t="str">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="C104" t="str">
-        <v>Chaitanya Jolly</v>
+        <v>Vidya poorna HS</v>
       </c>
       <c r="D104" t="str">
         <v>Bed A</v>
       </c>
       <c r="E104" t="str">
-        <v>8146762236</v>
+        <v>9663491347</v>
       </c>
       <c r="F104" t="str">
         <v>Single</v>
@@ -5596,10 +5596,10 @@
         <v>Tenant</v>
       </c>
       <c r="J104" t="str">
-        <v>08 Mar 2026</v>
+        <v>01 Nov 2025</v>
       </c>
       <c r="K104">
-        <v>20500</v>
+        <v>19000</v>
       </c>
       <c r="L104">
         <v>1</v>
@@ -5622,16 +5622,16 @@
         <v>104</v>
       </c>
       <c r="B105" t="str">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="C105" t="str">
-        <v>Pranjal Kumar</v>
+        <v>Chaitanya Jolly</v>
       </c>
       <c r="D105" t="str">
         <v>Bed A</v>
       </c>
       <c r="E105" t="str">
-        <v>7667539762</v>
+        <v>8146762236</v>
       </c>
       <c r="F105" t="str">
         <v>Single</v>
@@ -5646,10 +5646,10 @@
         <v>Tenant</v>
       </c>
       <c r="J105" t="str">
-        <v>01 Apr 2026</v>
+        <v>08 Mar 2026</v>
       </c>
       <c r="K105">
-        <v>18000</v>
+        <v>20500</v>
       </c>
       <c r="L105">
         <v>1</v>
@@ -5672,16 +5672,16 @@
         <v>105</v>
       </c>
       <c r="B106" t="str">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C106" t="str">
-        <v xml:space="preserve">Vaishnavi Deshpande </v>
+        <v>Pranjal Kumar</v>
       </c>
       <c r="D106" t="str">
         <v>Bed A</v>
       </c>
       <c r="E106" t="str">
-        <v>7799374327</v>
+        <v>7667539762</v>
       </c>
       <c r="F106" t="str">
         <v>Single</v>
@@ -5696,10 +5696,10 @@
         <v>Tenant</v>
       </c>
       <c r="J106" t="str">
-        <v>01 Feb 2026</v>
+        <v>01 Apr 2026</v>
       </c>
       <c r="K106">
-        <v>19900</v>
+        <v>18000</v>
       </c>
       <c r="L106">
         <v>1</v>
@@ -5722,19 +5722,19 @@
         <v>106</v>
       </c>
       <c r="B107" t="str">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C107" t="str">
-        <v>Anirudh Sridhar</v>
+        <v xml:space="preserve">Vaishnavi Deshpande </v>
       </c>
       <c r="D107" t="str">
         <v>Bed A</v>
       </c>
       <c r="E107" t="str">
-        <v>9687283596</v>
+        <v>7799374327</v>
       </c>
       <c r="F107" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G107" t="str">
         <v/>
@@ -5746,10 +5746,10 @@
         <v>Tenant</v>
       </c>
       <c r="J107" t="str">
-        <v>01 Jul 2026</v>
+        <v>01 Feb 2026</v>
       </c>
       <c r="K107">
-        <v>11000</v>
+        <v>19900</v>
       </c>
       <c r="L107">
         <v>1</v>
@@ -5775,13 +5775,13 @@
         <v>512</v>
       </c>
       <c r="C108" t="str">
-        <v>Shreya</v>
+        <v>Anirudh Sridhar</v>
       </c>
       <c r="D108" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E108" t="str">
-        <v>9108490448</v>
+        <v>9687283596</v>
       </c>
       <c r="F108" t="str">
         <v>2-Sharing</v>
@@ -5822,19 +5822,19 @@
         <v>108</v>
       </c>
       <c r="B109" t="str">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C109" t="str">
-        <v>Abhit Pandey</v>
+        <v>Shreya</v>
       </c>
       <c r="D109" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E109" t="str">
-        <v>9369688608</v>
+        <v>9108490448</v>
       </c>
       <c r="F109" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G109" t="str">
         <v/>
@@ -5846,10 +5846,10 @@
         <v>Tenant</v>
       </c>
       <c r="J109" t="str">
-        <v>28 Dec 2025</v>
+        <v>01 Jul 2026</v>
       </c>
       <c r="K109">
-        <v>17500</v>
+        <v>11000</v>
       </c>
       <c r="L109">
         <v>1</v>
@@ -5864,7 +5864,7 @@
         <v>0</v>
       </c>
       <c r="P109" t="str">
-        <v>KA13EQ3441</v>
+        <v/>
       </c>
     </row>
     <row r="110">
@@ -5872,19 +5872,19 @@
         <v>109</v>
       </c>
       <c r="B110" t="str">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="C110" t="str">
-        <v>Akilesh</v>
+        <v>Abhit Pandey</v>
       </c>
       <c r="D110" t="str">
         <v>Bed A</v>
       </c>
       <c r="E110" t="str">
-        <v>9705306559</v>
+        <v>9369688608</v>
       </c>
       <c r="F110" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G110" t="str">
         <v/>
@@ -5896,10 +5896,10 @@
         <v>Tenant</v>
       </c>
       <c r="J110" t="str">
-        <v>01 Oct 2026</v>
+        <v>28 Dec 2025</v>
       </c>
       <c r="K110">
-        <v>11000</v>
+        <v>17500</v>
       </c>
       <c r="L110">
         <v>1</v>
@@ -5914,7 +5914,7 @@
         <v>0</v>
       </c>
       <c r="P110" t="str">
-        <v/>
+        <v>KA13EQ3441</v>
       </c>
     </row>
     <row r="111">
@@ -5925,13 +5925,13 @@
         <v>514</v>
       </c>
       <c r="C111" t="str">
-        <v>Divyanshu Pandey</v>
+        <v>Akilesh</v>
       </c>
       <c r="D111" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E111" t="str">
-        <v>8797631089</v>
+        <v>9705306559</v>
       </c>
       <c r="F111" t="str">
         <v>2-Sharing</v>
@@ -5972,16 +5972,16 @@
         <v>111</v>
       </c>
       <c r="B112" t="str">
-        <v>601</v>
+        <v>514</v>
       </c>
       <c r="C112" t="str">
-        <v>Rajesh Kumar</v>
+        <v>Divyanshu Pandey</v>
       </c>
       <c r="D112" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E112" t="str">
-        <v>9063374806</v>
+        <v>8797631089</v>
       </c>
       <c r="F112" t="str">
         <v>2-Sharing</v>
@@ -5996,10 +5996,10 @@
         <v>Tenant</v>
       </c>
       <c r="J112" t="str">
-        <v>05 Oct 2026</v>
+        <v>01 Oct 2026</v>
       </c>
       <c r="K112">
-        <v>8000</v>
+        <v>11000</v>
       </c>
       <c r="L112">
         <v>1</v>
@@ -6025,13 +6025,13 @@
         <v>601</v>
       </c>
       <c r="C113" t="str">
-        <v>Vijay Akash</v>
+        <v>Rajesh Kumar</v>
       </c>
       <c r="D113" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E113" t="str">
-        <v>8248724588</v>
+        <v>9063374806</v>
       </c>
       <c r="F113" t="str">
         <v>2-Sharing</v>
@@ -6046,7 +6046,7 @@
         <v>Tenant</v>
       </c>
       <c r="J113" t="str">
-        <v>18 Oct 2026</v>
+        <v>05 Oct 2026</v>
       </c>
       <c r="K113">
         <v>8000</v>
@@ -6072,19 +6072,19 @@
         <v>113</v>
       </c>
       <c r="B114" t="str">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="C114" t="str">
-        <v>Harish Moorthy</v>
+        <v>Vijay Akash</v>
       </c>
       <c r="D114" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E114" t="str">
-        <v>8939529531</v>
+        <v>8248724588</v>
       </c>
       <c r="F114" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G114" t="str">
         <v/>
@@ -6096,10 +6096,10 @@
         <v>Tenant</v>
       </c>
       <c r="J114" t="str">
-        <v>01 Jan 2026</v>
+        <v>18 Oct 2026</v>
       </c>
       <c r="K114">
-        <v>20000</v>
+        <v>8000</v>
       </c>
       <c r="L114">
         <v>1</v>
@@ -6122,19 +6122,19 @@
         <v>114</v>
       </c>
       <c r="B115" t="str">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C115" t="str">
-        <v>Ravindra Reddy</v>
+        <v>Harish Moorthy</v>
       </c>
       <c r="D115" t="str">
         <v>Bed A</v>
       </c>
       <c r="E115" t="str">
-        <v>6362835867</v>
+        <v>8939529531</v>
       </c>
       <c r="F115" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G115" t="str">
         <v/>
@@ -6146,10 +6146,10 @@
         <v>Tenant</v>
       </c>
       <c r="J115" t="str">
-        <v>02 Sep 2026</v>
+        <v>01 Jan 2026</v>
       </c>
       <c r="K115">
-        <v>11000</v>
+        <v>20000</v>
       </c>
       <c r="L115">
         <v>1</v>
@@ -6175,13 +6175,13 @@
         <v>603</v>
       </c>
       <c r="C116" t="str">
-        <v>Praveen Sai</v>
+        <v>Ravindra Reddy</v>
       </c>
       <c r="D116" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E116" t="str">
-        <v>6303713939</v>
+        <v>6362835867</v>
       </c>
       <c r="F116" t="str">
         <v>2-Sharing</v>
@@ -6196,7 +6196,7 @@
         <v>Tenant</v>
       </c>
       <c r="J116" t="str">
-        <v>01 Oct 2026</v>
+        <v>02 Sep 2026</v>
       </c>
       <c r="K116">
         <v>11000</v>
@@ -6214,7 +6214,7 @@
         <v>0</v>
       </c>
       <c r="P116" t="str">
-        <v>AP40LH4400</v>
+        <v/>
       </c>
     </row>
     <row r="117">
@@ -6222,19 +6222,19 @@
         <v>116</v>
       </c>
       <c r="B117" t="str">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C117" t="str">
-        <v>Balamurali</v>
+        <v>Praveen Sai</v>
       </c>
       <c r="D117" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E117" t="str">
-        <v>9605062619</v>
+        <v>6303713939</v>
       </c>
       <c r="F117" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G117" t="str">
         <v/>
@@ -6246,10 +6246,10 @@
         <v>Tenant</v>
       </c>
       <c r="J117" t="str">
-        <v>08 Mar 2026</v>
+        <v>01 Oct 2026</v>
       </c>
       <c r="K117">
-        <v>21000</v>
+        <v>11000</v>
       </c>
       <c r="L117">
         <v>1</v>
@@ -6264,7 +6264,7 @@
         <v>0</v>
       </c>
       <c r="P117" t="str">
-        <v>KL01CN5887</v>
+        <v>AP40LH4400</v>
       </c>
     </row>
     <row r="118">
@@ -6272,19 +6272,19 @@
         <v>117</v>
       </c>
       <c r="B118" t="str">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="C118" t="str">
-        <v>Aditya Nandan</v>
+        <v>Balamurali</v>
       </c>
       <c r="D118" t="str">
         <v>Bed A</v>
       </c>
       <c r="E118" t="str">
-        <v>9955346752</v>
+        <v>9605062619</v>
       </c>
       <c r="F118" t="str">
-        <v>3-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G118" t="str">
         <v/>
@@ -6296,10 +6296,10 @@
         <v>Tenant</v>
       </c>
       <c r="J118" t="str">
-        <v>15 Aug 2026</v>
+        <v>08 Mar 2026</v>
       </c>
       <c r="K118">
-        <v>9000</v>
+        <v>21000</v>
       </c>
       <c r="L118">
         <v>1</v>
@@ -6314,7 +6314,7 @@
         <v>0</v>
       </c>
       <c r="P118" t="str">
-        <v/>
+        <v>KL01CN5887</v>
       </c>
     </row>
     <row r="119">
@@ -6325,13 +6325,13 @@
         <v>605</v>
       </c>
       <c r="C119" t="str">
-        <v>Siva Krishna</v>
+        <v>Aditya Nandan</v>
       </c>
       <c r="D119" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E119" t="str">
-        <v>8608233665</v>
+        <v>9955346752</v>
       </c>
       <c r="F119" t="str">
         <v>3-Sharing</v>
@@ -6346,10 +6346,10 @@
         <v>Tenant</v>
       </c>
       <c r="J119" t="str">
-        <v>28 Nov 2025</v>
+        <v>15 Aug 2026</v>
       </c>
       <c r="K119">
-        <v>8000</v>
+        <v>9000</v>
       </c>
       <c r="L119">
         <v>1</v>
@@ -6375,13 +6375,13 @@
         <v>605</v>
       </c>
       <c r="C120" t="str">
-        <v>Dundigala Sravan</v>
+        <v>Siva Krishna</v>
       </c>
       <c r="D120" t="str">
-        <v>Bed C</v>
+        <v>Bed B</v>
       </c>
       <c r="E120" t="str">
-        <v>6300294014</v>
+        <v>8608233665</v>
       </c>
       <c r="F120" t="str">
         <v>3-Sharing</v>
@@ -6396,7 +6396,7 @@
         <v>Tenant</v>
       </c>
       <c r="J120" t="str">
-        <v>09 Sep 2026</v>
+        <v>28 Nov 2025</v>
       </c>
       <c r="K120">
         <v>8000</v>
@@ -6422,19 +6422,19 @@
         <v>120</v>
       </c>
       <c r="B121" t="str">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C121" t="str">
-        <v>Palak</v>
+        <v>Dundigala Sravan</v>
       </c>
       <c r="D121" t="str">
-        <v>Bed A</v>
+        <v>Bed C</v>
       </c>
       <c r="E121" t="str">
-        <v>9556210524</v>
+        <v>6300294014</v>
       </c>
       <c r="F121" t="str">
-        <v>Single</v>
+        <v>3-Sharing</v>
       </c>
       <c r="G121" t="str">
         <v/>
@@ -6446,10 +6446,10 @@
         <v>Tenant</v>
       </c>
       <c r="J121" t="str">
-        <v>25 Sep 2026</v>
+        <v>09 Sep 2026</v>
       </c>
       <c r="K121">
-        <v>19000</v>
+        <v>8000</v>
       </c>
       <c r="L121">
         <v>1</v>
@@ -6472,16 +6472,16 @@
         <v>121</v>
       </c>
       <c r="B122" t="str">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="C122" t="str">
-        <v>Aryan</v>
+        <v>Palak</v>
       </c>
       <c r="D122" t="str">
         <v>Bed A</v>
       </c>
       <c r="E122" t="str">
-        <v>9406501415</v>
+        <v>9556210524</v>
       </c>
       <c r="F122" t="str">
         <v>Single</v>
@@ -6496,10 +6496,10 @@
         <v>Tenant</v>
       </c>
       <c r="J122" t="str">
-        <v>02 Jul 2026</v>
+        <v>25 Sep 2026</v>
       </c>
       <c r="K122">
-        <v>20000</v>
+        <v>19000</v>
       </c>
       <c r="L122">
         <v>1</v>
@@ -6522,16 +6522,16 @@
         <v>122</v>
       </c>
       <c r="B123" t="str">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="C123" t="str">
-        <v>Srinath</v>
+        <v>Aryan</v>
       </c>
       <c r="D123" t="str">
         <v>Bed A</v>
       </c>
       <c r="E123" t="str">
-        <v>7396249645</v>
+        <v>9406501415</v>
       </c>
       <c r="F123" t="str">
         <v>Single</v>
@@ -6546,10 +6546,10 @@
         <v>Tenant</v>
       </c>
       <c r="J123" t="str">
-        <v>03 Dec 2025</v>
+        <v>02 Jul 2026</v>
       </c>
       <c r="K123">
-        <v>11000</v>
+        <v>20000</v>
       </c>
       <c r="L123">
         <v>1</v>
@@ -6572,19 +6572,19 @@
         <v>123</v>
       </c>
       <c r="B124" t="str">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="C124" t="str">
-        <v>Neemkar Amarnath Rao</v>
+        <v>Srinath</v>
       </c>
       <c r="D124" t="str">
         <v>Bed A</v>
       </c>
       <c r="E124" t="str">
-        <v>8520860144</v>
+        <v>7396249645</v>
       </c>
       <c r="F124" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G124" t="str">
         <v/>
@@ -6596,13 +6596,13 @@
         <v>Tenant</v>
       </c>
       <c r="J124" t="str">
-        <v>01 Feb 2026</v>
+        <v>03 Dec 2025</v>
       </c>
       <c r="K124">
-        <v>18500</v>
+        <v>11000</v>
       </c>
       <c r="L124">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M124" t="str">
         <v>Yes (Paid)</v>
@@ -6622,19 +6622,19 @@
         <v>124</v>
       </c>
       <c r="B125" t="str">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="C125" t="str">
-        <v>Dharya</v>
+        <v>DINESH KUMAR</v>
       </c>
       <c r="D125" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E125" t="str">
-        <v>9484665330</v>
+        <v>7449102846</v>
       </c>
       <c r="F125" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G125" t="str">
         <v/>
@@ -6646,13 +6646,13 @@
         <v>Tenant</v>
       </c>
       <c r="J125" t="str">
-        <v>26 Mar 2026</v>
+        <v>31 Oct 2026</v>
       </c>
       <c r="K125">
-        <v>17500</v>
+        <v>11000</v>
       </c>
       <c r="L125">
-        <v>1</v>
+        <v>5000</v>
       </c>
       <c r="M125" t="str">
         <v>Yes (Paid)</v>
@@ -6672,19 +6672,19 @@
         <v>125</v>
       </c>
       <c r="B126" t="str">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="C126" t="str">
-        <v>Anuroop Sadashiv</v>
+        <v>Neemkar Amarnath Rao</v>
       </c>
       <c r="D126" t="str">
         <v>Bed A</v>
       </c>
       <c r="E126" t="str">
-        <v>9967940815</v>
+        <v>8520860144</v>
       </c>
       <c r="F126" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G126" t="str">
         <v/>
@@ -6696,13 +6696,13 @@
         <v>Tenant</v>
       </c>
       <c r="J126" t="str">
-        <v>05 Jan 2026</v>
+        <v>01 Feb 2026</v>
       </c>
       <c r="K126">
-        <v>11000</v>
+        <v>18500</v>
       </c>
       <c r="L126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M126" t="str">
         <v>Yes (Paid)</v>
@@ -6722,19 +6722,19 @@
         <v>126</v>
       </c>
       <c r="B127" t="str">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="C127" t="str">
-        <v>Sai teja</v>
+        <v>Dharya</v>
       </c>
       <c r="D127" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E127" t="str">
-        <v>9293399888</v>
+        <v>9484665330</v>
       </c>
       <c r="F127" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G127" t="str">
         <v/>
@@ -6746,10 +6746,10 @@
         <v>Tenant</v>
       </c>
       <c r="J127" t="str">
-        <v>04 Jan 2026</v>
+        <v>26 Mar 2026</v>
       </c>
       <c r="K127">
-        <v>11000</v>
+        <v>17500</v>
       </c>
       <c r="L127">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>0</v>
       </c>
       <c r="P127" t="str">
-        <v>TS03FB8844</v>
+        <v/>
       </c>
     </row>
     <row r="128">
@@ -6772,16 +6772,16 @@
         <v>127</v>
       </c>
       <c r="B128" t="str">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="C128" t="str">
-        <v>Shiva</v>
+        <v>Anuroop Sadashiv</v>
       </c>
       <c r="D128" t="str">
         <v>Bed A</v>
       </c>
       <c r="E128" t="str">
-        <v>9632761194</v>
+        <v>9967940815</v>
       </c>
       <c r="F128" t="str">
         <v>2-Sharing</v>
@@ -6796,7 +6796,7 @@
         <v>Tenant</v>
       </c>
       <c r="J128" t="str">
-        <v>01 Oct 2026</v>
+        <v>05 Jan 2026</v>
       </c>
       <c r="K128">
         <v>11000</v>
@@ -6814,7 +6814,7 @@
         <v>0</v>
       </c>
       <c r="P128" t="str">
-        <v>KA53HT5130</v>
+        <v/>
       </c>
     </row>
     <row r="129">
@@ -6822,16 +6822,16 @@
         <v>128</v>
       </c>
       <c r="B129" t="str">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="C129" t="str">
-        <v>Manoj Veerabhadra</v>
+        <v>Sai teja</v>
       </c>
       <c r="D129" t="str">
         <v>Bed B</v>
       </c>
       <c r="E129" t="str">
-        <v>7989522145</v>
+        <v>9293399888</v>
       </c>
       <c r="F129" t="str">
         <v>2-Sharing</v>
@@ -6846,7 +6846,7 @@
         <v>Tenant</v>
       </c>
       <c r="J129" t="str">
-        <v>01 Nov 2025</v>
+        <v>04 Jan 2026</v>
       </c>
       <c r="K129">
         <v>11000</v>
@@ -6864,7 +6864,7 @@
         <v>0</v>
       </c>
       <c r="P129" t="str">
-        <v>KA03LJ6820</v>
+        <v>TS03FB8844</v>
       </c>
     </row>
     <row r="130">
@@ -6872,19 +6872,19 @@
         <v>129</v>
       </c>
       <c r="B130" t="str">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="C130" t="str">
-        <v>Kalandar</v>
+        <v>Shiva</v>
       </c>
       <c r="D130" t="str">
         <v>Bed A</v>
       </c>
       <c r="E130" t="str">
-        <v>7899567998</v>
+        <v>9632761194</v>
       </c>
       <c r="F130" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G130" t="str">
         <v/>
@@ -6896,10 +6896,10 @@
         <v>Tenant</v>
       </c>
       <c r="J130" t="str">
-        <v>01 Jan 2026</v>
+        <v>01 Oct 2026</v>
       </c>
       <c r="K130">
-        <v>18000</v>
+        <v>11000</v>
       </c>
       <c r="L130">
         <v>1</v>
@@ -6914,7 +6914,7 @@
         <v>0</v>
       </c>
       <c r="P130" t="str">
-        <v>KA21EA3750</v>
+        <v>KA53HT5130</v>
       </c>
     </row>
     <row r="131">
@@ -6922,16 +6922,16 @@
         <v>130</v>
       </c>
       <c r="B131" t="str">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C131" t="str">
-        <v>P Akilesh Pattani Raman</v>
+        <v>Manoj Veerabhadra</v>
       </c>
       <c r="D131" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E131" t="str">
-        <v>9398815361</v>
+        <v>7989522145</v>
       </c>
       <c r="F131" t="str">
         <v>2-Sharing</v>
@@ -6946,7 +6946,7 @@
         <v>Tenant</v>
       </c>
       <c r="J131" t="str">
-        <v>01 Jun 2026</v>
+        <v>01 Nov 2025</v>
       </c>
       <c r="K131">
         <v>11000</v>
@@ -6964,7 +6964,7 @@
         <v>0</v>
       </c>
       <c r="P131" t="str">
-        <v/>
+        <v>KA03LJ6820</v>
       </c>
     </row>
     <row r="132">
@@ -6972,19 +6972,19 @@
         <v>131</v>
       </c>
       <c r="B132" t="str">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="C132" t="str">
-        <v>Viraj Bontha</v>
+        <v>Kalandar</v>
       </c>
       <c r="D132" t="str">
-        <v>Bed B</v>
+        <v>Bed A</v>
       </c>
       <c r="E132" t="str">
-        <v>6281122607</v>
+        <v>7899567998</v>
       </c>
       <c r="F132" t="str">
-        <v>2-Sharing</v>
+        <v>Single</v>
       </c>
       <c r="G132" t="str">
         <v/>
@@ -6996,10 +6996,10 @@
         <v>Tenant</v>
       </c>
       <c r="J132" t="str">
-        <v>18 Jan 2026</v>
+        <v>01 Jan 2026</v>
       </c>
       <c r="K132">
-        <v>11000</v>
+        <v>18000</v>
       </c>
       <c r="L132">
         <v>1</v>
@@ -7014,7 +7014,7 @@
         <v>0</v>
       </c>
       <c r="P132" t="str">
-        <v/>
+        <v>KA21EA3750</v>
       </c>
     </row>
     <row r="133">
@@ -7022,16 +7022,16 @@
         <v>132</v>
       </c>
       <c r="B133" t="str">
-        <v>701</v>
+        <v>614</v>
       </c>
       <c r="C133" t="str">
-        <v>Chakravarti</v>
+        <v>P Akilesh Pattani Raman</v>
       </c>
       <c r="D133" t="str">
         <v>Bed A</v>
       </c>
       <c r="E133" t="str">
-        <v>8688094388</v>
+        <v>9398815361</v>
       </c>
       <c r="F133" t="str">
         <v>2-Sharing</v>
@@ -7046,10 +7046,10 @@
         <v>Tenant</v>
       </c>
       <c r="J133" t="str">
-        <v>04 Jan 2026</v>
+        <v>01 Jun 2026</v>
       </c>
       <c r="K133">
-        <v>11500</v>
+        <v>11000</v>
       </c>
       <c r="L133">
         <v>1</v>
@@ -7072,16 +7072,16 @@
         <v>133</v>
       </c>
       <c r="B134" t="str">
-        <v>701</v>
+        <v>614</v>
       </c>
       <c r="C134" t="str">
-        <v>Rohit</v>
+        <v>Viraj Bontha</v>
       </c>
       <c r="D134" t="str">
         <v>Bed B</v>
       </c>
       <c r="E134" t="str">
-        <v>9701884938</v>
+        <v>6281122607</v>
       </c>
       <c r="F134" t="str">
         <v>2-Sharing</v>
@@ -7096,10 +7096,10 @@
         <v>Tenant</v>
       </c>
       <c r="J134" t="str">
-        <v>04 Jan 2026</v>
+        <v>18 Jan 2026</v>
       </c>
       <c r="K134">
-        <v>11500</v>
+        <v>11000</v>
       </c>
       <c r="L134">
         <v>1</v>
@@ -7122,16 +7122,16 @@
         <v>134</v>
       </c>
       <c r="B135" t="str">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C135" t="str">
-        <v>Ashrith</v>
+        <v>Chakravarti</v>
       </c>
       <c r="D135" t="str">
         <v>Bed A</v>
       </c>
       <c r="E135" t="str">
-        <v>9652220621</v>
+        <v>8688094388</v>
       </c>
       <c r="F135" t="str">
         <v>2-Sharing</v>
@@ -7164,7 +7164,7 @@
         <v>0</v>
       </c>
       <c r="P135" t="str">
-        <v>AP21BW7154</v>
+        <v/>
       </c>
     </row>
     <row r="136">
@@ -7172,16 +7172,16 @@
         <v>135</v>
       </c>
       <c r="B136" t="str">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C136" t="str">
-        <v>Vivek Vardhan Reddy</v>
+        <v>Rohit</v>
       </c>
       <c r="D136" t="str">
         <v>Bed B</v>
       </c>
       <c r="E136" t="str">
-        <v>9110365970</v>
+        <v>9701884938</v>
       </c>
       <c r="F136" t="str">
         <v>2-Sharing</v>
@@ -7222,19 +7222,19 @@
         <v>136</v>
       </c>
       <c r="B137" t="str">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C137" t="str">
-        <v>S G Gopinath</v>
+        <v>Ashrith</v>
       </c>
       <c r="D137" t="str">
         <v>Bed A</v>
       </c>
       <c r="E137" t="str">
-        <v>9894548386</v>
+        <v>9652220621</v>
       </c>
       <c r="F137" t="str">
-        <v>Single</v>
+        <v>2-Sharing</v>
       </c>
       <c r="G137" t="str">
         <v/>
@@ -7246,10 +7246,10 @@
         <v>Tenant</v>
       </c>
       <c r="J137" t="str">
-        <v>01 Jan 2026</v>
+        <v>04 Jan 2026</v>
       </c>
       <c r="K137">
-        <v>11000</v>
+        <v>11500</v>
       </c>
       <c r="L137">
         <v>1</v>
@@ -7264,7 +7264,7 @@
         <v>0</v>
       </c>
       <c r="P137" t="str">
-        <v/>
+        <v>AP21BW7154</v>
       </c>
     </row>
     <row r="138">
@@ -7272,16 +7272,16 @@
         <v>137</v>
       </c>
       <c r="B138" t="str">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="C138" t="str">
-        <v>Chirag Yadav</v>
+        <v>Vivek Vardhan Reddy</v>
       </c>
       <c r="D138" t="str">
-        <v>Bed A</v>
+        <v>Bed B</v>
       </c>
       <c r="E138" t="str">
-        <v>8447573101</v>
+        <v>9110365970</v>
       </c>
       <c r="F138" t="str">
         <v>2-Sharing</v>
@@ -7296,10 +7296,10 @@
         <v>Tenant</v>
       </c>
       <c r="J138" t="str">
-        <v>30 Sep 2026</v>
+        <v>04 Jan 2026</v>
       </c>
       <c r="K138">
-        <v>9000</v>
+        <v>11500</v>
       </c>
       <c r="L138">
         <v>1</v>
@@ -7322,54 +7322,204 @@
         <v>138</v>
       </c>
       <c r="B139" t="str">
+        <v>703</v>
+      </c>
+      <c r="C139" t="str">
+        <v>S G Gopinath</v>
+      </c>
+      <c r="D139" t="str">
+        <v>Bed A</v>
+      </c>
+      <c r="E139" t="str">
+        <v>9894548386</v>
+      </c>
+      <c r="F139" t="str">
+        <v>Single</v>
+      </c>
+      <c r="G139" t="str">
+        <v/>
+      </c>
+      <c r="H139" t="str">
+        <v/>
+      </c>
+      <c r="I139" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="J139" t="str">
+        <v>01 Jan 2026</v>
+      </c>
+      <c r="K139">
+        <v>11000</v>
+      </c>
+      <c r="L139">
+        <v>1</v>
+      </c>
+      <c r="M139" t="str">
+        <v>Yes (Paid)</v>
+      </c>
+      <c r="N139" t="str">
+        <v>Yes (Paid)</v>
+      </c>
+      <c r="O139">
+        <v>0</v>
+      </c>
+      <c r="P139" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="str">
         <v>704</v>
       </c>
-      <c r="C139" t="str">
+      <c r="C140" t="str">
+        <v>Chirag Yadav</v>
+      </c>
+      <c r="D140" t="str">
+        <v>Bed A</v>
+      </c>
+      <c r="E140" t="str">
+        <v>8447573101</v>
+      </c>
+      <c r="F140" t="str">
+        <v>2-Sharing</v>
+      </c>
+      <c r="G140" t="str">
+        <v/>
+      </c>
+      <c r="H140" t="str">
+        <v/>
+      </c>
+      <c r="I140" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="J140" t="str">
+        <v>30 Sep 2026</v>
+      </c>
+      <c r="K140">
+        <v>9000</v>
+      </c>
+      <c r="L140">
+        <v>1</v>
+      </c>
+      <c r="M140" t="str">
+        <v>Yes (Paid)</v>
+      </c>
+      <c r="N140" t="str">
+        <v>Yes (Paid)</v>
+      </c>
+      <c r="O140">
+        <v>0</v>
+      </c>
+      <c r="P140" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="str">
+        <v>704</v>
+      </c>
+      <c r="C141" t="str">
         <v>Shaik Irfan</v>
       </c>
-      <c r="D139" t="str">
+      <c r="D141" t="str">
         <v>Bed B</v>
       </c>
-      <c r="E139" t="str">
+      <c r="E141" t="str">
         <v>6281008834</v>
       </c>
-      <c r="F139" t="str">
-        <v>2-Sharing</v>
-      </c>
-      <c r="G139" t="str">
-        <v/>
-      </c>
-      <c r="H139" t="str">
-        <v/>
-      </c>
-      <c r="I139" t="str">
-        <v>Tenant</v>
-      </c>
-      <c r="J139" t="str">
+      <c r="F141" t="str">
+        <v>2-Sharing</v>
+      </c>
+      <c r="G141" t="str">
+        <v/>
+      </c>
+      <c r="H141" t="str">
+        <v/>
+      </c>
+      <c r="I141" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="J141" t="str">
         <v>30 Sep 2026</v>
       </c>
-      <c r="K139">
+      <c r="K141">
         <v>9000</v>
       </c>
-      <c r="L139">
-        <v>1</v>
-      </c>
-      <c r="M139" t="str">
-        <v>Yes (Paid)</v>
-      </c>
-      <c r="N139" t="str">
-        <v>Yes (Paid)</v>
-      </c>
-      <c r="O139">
-        <v>0</v>
-      </c>
-      <c r="P139" t="str">
+      <c r="L141">
+        <v>1</v>
+      </c>
+      <c r="M141" t="str">
+        <v>Yes (Paid)</v>
+      </c>
+      <c r="N141" t="str">
+        <v>Yes (Paid)</v>
+      </c>
+      <c r="O141">
+        <v>0</v>
+      </c>
+      <c r="P141" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="str">
+        <v>GA</v>
+      </c>
+      <c r="C142" t="str">
+        <v>PG Management</v>
+      </c>
+      <c r="D142" t="str">
+        <v>Bed A</v>
+      </c>
+      <c r="E142" t="str">
+        <v>7090803339</v>
+      </c>
+      <c r="F142" t="str">
+        <v>Single</v>
+      </c>
+      <c r="G142" t="str">
+        <v/>
+      </c>
+      <c r="H142" t="str">
+        <v/>
+      </c>
+      <c r="I142" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="J142" t="str">
+        <v>01 Nov 2026</v>
+      </c>
+      <c r="K142">
+        <v>1</v>
+      </c>
+      <c r="L142">
+        <v>1</v>
+      </c>
+      <c r="M142" t="str">
+        <v>No (Due)</v>
+      </c>
+      <c r="N142" t="str">
+        <v>Yes (Paid)</v>
+      </c>
+      <c r="O142">
+        <v>0</v>
+      </c>
+      <c r="P142" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P139"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P142"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>